<commit_message>
avance graficos - solo falta 1 grafico de ptr
</commit_message>
<xml_diff>
--- a/Backend/Input/format_reports/formato.xlsx
+++ b/Backend/Input/format_reports/formato.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr filterPrivacy="1" hidePivotFieldList="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74A50B53-3119-40C9-B07B-CD69BE58A8A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43E610CC-5F20-4BA9-B71C-9E29B723268C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="0" windowWidth="21600" windowHeight="11295" tabRatio="719" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6240" yWindow="855" windowWidth="20460" windowHeight="10770" tabRatio="719" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portada" sheetId="52" r:id="rId1"/>
@@ -9768,8 +9768,8 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="4.4308759803029896E-2"/>
-          <c:y val="4.2570660733148004E-2"/>
+          <c:x val="4.8405549178221811E-2"/>
+          <c:y val="0"/>
           <c:w val="0.92839209892452568"/>
           <c:h val="0.87797396482705137"/>
         </c:manualLayout>
@@ -10128,6 +10128,14 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.10697682406354191"/>
+          <c:y val="4.1212112034207132E-2"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -10164,8 +10172,8 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="4.0125577630341101E-2"/>
-          <c:y val="0.22576923538662858"/>
+          <c:x val="5.4958833954806087E-2"/>
+          <c:y val="0.22576931318592031"/>
           <c:w val="0.91300096501850747"/>
           <c:h val="0.57180930885866232"/>
         </c:manualLayout>
@@ -14167,10 +14175,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="1.3060085544800641E-2"/>
-          <c:y val="2.9499386517305291E-2"/>
-          <c:w val="0.97318749094521595"/>
-          <c:h val="0.92741181102362202"/>
+          <c:x val="7.7842671480226888E-3"/>
+          <c:y val="9.2114234728880497E-3"/>
+          <c:w val="0.98905294856629578"/>
+          <c:h val="0.95418813441803541"/>
         </c:manualLayout>
       </c:layout>
       <c:barChart>
@@ -14435,7 +14443,7 @@
       </c:valAx>
       <c:spPr>
         <a:noFill/>
-        <a:ln>
+        <a:ln w="25400">
           <a:noFill/>
         </a:ln>
         <a:effectLst/>
@@ -27581,13 +27589,13 @@
       <xdr:col>5</xdr:col>
       <xdr:colOff>440379</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>294657</xdr:rowOff>
+      <xdr:rowOff>225384</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>467591</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>246847</xdr:rowOff>
+      <xdr:rowOff>177574</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -27602,7 +27610,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6744197" y="5559384"/>
+          <a:off x="6744197" y="5490111"/>
           <a:ext cx="6261758" cy="437099"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -27660,13 +27668,13 @@
       <xdr:col>12</xdr:col>
       <xdr:colOff>622218</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>283971</xdr:rowOff>
+      <xdr:rowOff>232017</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>5645728</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>218949</xdr:rowOff>
+      <xdr:rowOff>166995</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -27681,7 +27689,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13160582" y="5548698"/>
+          <a:off x="13160582" y="5496744"/>
           <a:ext cx="9612828" cy="419887"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -27754,15 +27762,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>350076</xdr:colOff>
+      <xdr:colOff>277091</xdr:colOff>
       <xdr:row>32</xdr:row>
-      <xdr:rowOff>178131</xdr:rowOff>
+      <xdr:rowOff>34636</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>439140</xdr:colOff>
+      <xdr:colOff>421821</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>178130</xdr:rowOff>
+      <xdr:rowOff>22265</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -27777,8 +27785,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6653894" y="10620995"/>
-          <a:ext cx="6323610" cy="380999"/>
+          <a:off x="6580909" y="10477500"/>
+          <a:ext cx="6379276" cy="368629"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -27833,15 +27841,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>623454</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>-1</xdr:rowOff>
+      <xdr:colOff>640772</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>34636</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>5559136</xdr:colOff>
+      <xdr:colOff>5645727</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>173182</xdr:rowOff>
+      <xdr:rowOff>17319</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -27856,8 +27864,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13161818" y="10633363"/>
-          <a:ext cx="9525000" cy="363683"/>
+          <a:off x="13179136" y="10477500"/>
+          <a:ext cx="9594273" cy="363683"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -27913,14 +27921,14 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>450273</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>51955</xdr:rowOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>259774</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>467591</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>467592</xdr:rowOff>
+      <xdr:colOff>381001</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>69271</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -27954,14 +27962,14 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>311727</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>69272</xdr:rowOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>155864</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>415637</xdr:colOff>
       <xdr:row>50</xdr:row>
-      <xdr:rowOff>51953</xdr:rowOff>
+      <xdr:rowOff>51954</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -28265,9 +28273,9 @@
       <xdr:rowOff>329046</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>27</xdr:row>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>5628409</xdr:colOff>
+      <xdr:row>30</xdr:row>
       <xdr:rowOff>17318</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -28301,15 +28309,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>606136</xdr:colOff>
+      <xdr:colOff>640772</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>69273</xdr:rowOff>
+      <xdr:rowOff>17317</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>5583584</xdr:colOff>
+      <xdr:colOff>5645727</xdr:colOff>
       <xdr:row>50</xdr:row>
-      <xdr:rowOff>69273</xdr:rowOff>
+      <xdr:rowOff>86590</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -29711,7 +29719,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s313200"/>
+                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s327222"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29776,7 +29784,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s313201"/>
+                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s327223"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29893,7 +29901,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$6:$C$10" spid="_x0000_s313202"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$6:$C$10" spid="_x0000_s327224"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29958,7 +29966,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$11:$C$14" spid="_x0000_s313203"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$11:$C$14" spid="_x0000_s327225"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -30023,7 +30031,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$15:$C$18" spid="_x0000_s313204"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$15:$C$18" spid="_x0000_s327226"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -30088,7 +30096,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$19:$C$26" spid="_x0000_s313205"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$19:$C$26" spid="_x0000_s327227"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -30153,7 +30161,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$27:$C$32" spid="_x0000_s313206"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$27:$C$32" spid="_x0000_s327228"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -30218,7 +30226,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$33:$C$39" spid="_x0000_s313207"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$33:$C$39" spid="_x0000_s327229"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -30283,7 +30291,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$40:$C$46" spid="_x0000_s313208"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$40:$C$46" spid="_x0000_s327230"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -30348,7 +30356,7 @@
               <a:picLocks noChangeAspect="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$3:$C$5" spid="_x0000_s313209"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$3:$C$5" spid="_x0000_s327231"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -33094,7 +33102,7 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="14" name="Gráfico 13">
+        <xdr:cNvPr id="14" name="signals_chart">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25950EC3-1590-32C4-829D-B644D554DDF0}"/>
@@ -33118,19 +33126,19 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>44822</xdr:colOff>
+      <xdr:colOff>717176</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>291354</xdr:rowOff>
+      <xdr:rowOff>112059</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>235323</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1008529</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>44824</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="15" name="Gráfico 14">
+        <xdr:cNvPr id="15" name="ptr_chart">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{44FBD140-EB46-B47C-FF82-ACD6C1641FD5}"/>

</xml_diff>

<commit_message>
se corrigen errores de rutas y se unifica la extacción de datos con la eleboración del informe
</commit_message>
<xml_diff>
--- a/Backend/Input/format_reports/formato.xlsx
+++ b/Backend/Input/format_reports/formato.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr filterPrivacy="1" hidePivotFieldList="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77263F2E-038A-4143-B0B5-FFD96533B3AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00297E93-2A58-4D44-BF89-21DE2E91BD42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7965" yWindow="1395" windowWidth="15015" windowHeight="12210" tabRatio="719" firstSheet="12" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7380" yWindow="0" windowWidth="21525" windowHeight="11295" tabRatio="719" firstSheet="12" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portada" sheetId="52" r:id="rId1"/>
@@ -29463,7 +29463,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s341434"/>
+                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s341654"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29528,7 +29528,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s341435"/>
+                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s341655"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29645,7 +29645,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$6:$C$10" spid="_x0000_s341436"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$6:$C$10" spid="_x0000_s341656"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29710,7 +29710,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$11:$C$14" spid="_x0000_s341437"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$11:$C$14" spid="_x0000_s341657"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29775,7 +29775,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$15:$C$18" spid="_x0000_s341438"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$15:$C$18" spid="_x0000_s341658"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29840,7 +29840,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$19:$C$26" spid="_x0000_s341439"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$19:$C$26" spid="_x0000_s341659"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29905,7 +29905,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$27:$C$32" spid="_x0000_s341440"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$27:$C$32" spid="_x0000_s341660"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -29970,7 +29970,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$33:$C$39" spid="_x0000_s341441"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$33:$C$39" spid="_x0000_s341661"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -30035,7 +30035,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$40:$C$46" spid="_x0000_s341442"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$40:$C$46" spid="_x0000_s341662"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -30100,7 +30100,7 @@
               <a:picLocks noChangeAspect="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$3:$C$5" spid="_x0000_s341443"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$3:$C$5" spid="_x0000_s341663"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -44009,7 +44009,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="5" scale="50" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="5" scale="51" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="51" max="18" man="1"/>
   </rowBreaks>

</xml_diff>

<commit_message>
se corrige, error en el orden de descargar y guardado de archivos y planillas
</commit_message>
<xml_diff>
--- a/Backend/Input/format_reports/formato.xlsx
+++ b/Backend/Input/format_reports/formato.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr filterPrivacy="1" hidePivotFieldList="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B6B6C8-9ED8-4B7A-8D02-CB699EC0B708}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CAF7192-60B9-4711-8C50-761B1DA6ED59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="719" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="719" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portada" sheetId="52" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="Convenios ADP_II" sheetId="54" state="hidden" r:id="rId10"/>
     <sheet name="Gestión de riesgos" sheetId="48" r:id="rId11"/>
     <sheet name="data_riesgos" sheetId="49" state="hidden" r:id="rId12"/>
-    <sheet name="Planes de tratamientos" sheetId="55" r:id="rId13"/>
+    <sheet name="Planes de tratamientos" sheetId="55" state="hidden" r:id="rId13"/>
     <sheet name="Planes tratamientos" sheetId="53" state="hidden" r:id="rId14"/>
   </sheets>
   <definedNames>
@@ -9270,6 +9270,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9277,7 +9278,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9663,6 +9663,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9670,7 +9671,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -9883,6 +9883,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -9890,7 +9891,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10103,6 +10103,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10110,7 +10111,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -10676,6 +10676,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -10683,7 +10684,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11013,6 +11013,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -11020,7 +11021,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11342,6 +11342,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -11349,7 +11350,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11685,6 +11685,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -11692,7 +11693,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -12871,6 +12871,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -12878,7 +12879,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -14048,6 +14048,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -14055,7 +14056,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -15002,6 +15002,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -15009,7 +15010,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:noFill/>
@@ -15526,6 +15526,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -15533,7 +15534,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -15890,6 +15890,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -15897,7 +15898,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -25550,7 +25550,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s382782"/>
+                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s382922"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -25615,7 +25615,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s382783"/>
+                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s382923"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -25732,7 +25732,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$6:$C$10" spid="_x0000_s382784"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$6:$C$10" spid="_x0000_s382924"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -25797,7 +25797,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$11:$C$14" spid="_x0000_s382785"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$11:$C$14" spid="_x0000_s382925"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -25862,7 +25862,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$15:$C$18" spid="_x0000_s382786"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$15:$C$18" spid="_x0000_s382926"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -25927,7 +25927,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$19:$C$26" spid="_x0000_s382787"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$19:$C$26" spid="_x0000_s382927"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -25992,7 +25992,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$27:$C$32" spid="_x0000_s382788"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$27:$C$32" spid="_x0000_s382928"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -26057,7 +26057,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$33:$C$39" spid="_x0000_s382789"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$33:$C$39" spid="_x0000_s382929"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -26122,7 +26122,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$40:$C$46" spid="_x0000_s382790"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$40:$C$46" spid="_x0000_s382930"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -26187,7 +26187,7 @@
               <a:picLocks noChangeAspect="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$3:$C$5" spid="_x0000_s382791"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$3:$C$5" spid="_x0000_s382931"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -38909,7 +38909,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="5" scale="50" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="5" scale="51" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="51" max="18" man="1"/>
   </rowBreaks>

</xml_diff>

<commit_message>
penultimo avance 05-08-2025;1:21 am
</commit_message>
<xml_diff>
--- a/Backend/Input/format_reports/formato.xlsx
+++ b/Backend/Input/format_reports/formato.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr filterPrivacy="1" hidePivotFieldList="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CAF7192-60B9-4711-8C50-761B1DA6ED59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBC7EBB6-E908-4A87-A2A5-8D8280959CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="719" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="719" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portada" sheetId="52" r:id="rId1"/>
@@ -25550,7 +25550,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s382922"/>
+                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s394286"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -25615,7 +25615,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s382923"/>
+                  <a14:cameraTool cellRange="data_status_NC!#REF!" spid="_x0000_s394287"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -25732,7 +25732,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$6:$C$10" spid="_x0000_s382924"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$6:$C$10" spid="_x0000_s394288"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -25797,7 +25797,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$11:$C$14" spid="_x0000_s382925"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$11:$C$14" spid="_x0000_s394289"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -25862,7 +25862,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$15:$C$18" spid="_x0000_s382926"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$15:$C$18" spid="_x0000_s394290"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -25927,7 +25927,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$19:$C$26" spid="_x0000_s382927"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$19:$C$26" spid="_x0000_s394291"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -25992,7 +25992,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$27:$C$32" spid="_x0000_s382928"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$27:$C$32" spid="_x0000_s394292"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -26057,7 +26057,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$33:$C$39" spid="_x0000_s382929"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$33:$C$39" spid="_x0000_s394293"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -26122,7 +26122,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$40:$C$46" spid="_x0000_s382930"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$40:$C$46" spid="_x0000_s394294"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -26187,7 +26187,7 @@
               <a:picLocks noChangeAspect="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="data_status_NC!$B$3:$C$5" spid="_x0000_s382931"/>
+                  <a14:cameraTool cellRange="data_status_NC!$B$3:$C$5" spid="_x0000_s394295"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>

</xml_diff>